<commit_message>
Update 26-01-2026: Acortados nombres carpetas y fusionados scripts de limpieza ENFR y proyecciones poblacionales, creado script con simulaciones AVP, AVD, AVAD y tasas
</commit_message>
<xml_diff>
--- a/datos_limpios/dic_arg_dm2_ge10.xlsx
+++ b/datos_limpios/dic_arg_dm2_ge10.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -621,12 +621,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dm2_prev</t>
+          <t>dm_prev</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Prevalencia de DM2 por provincia, grupo etario y sexo</t>
+          <t>Prevalencia de DM por provincia, grupo etario y sexo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dm2_prev_se</t>
+          <t>dm_prev_se</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Error estándar del total de la prevalencia de personas con DM2</t>
+          <t>Error estándar del total de la prevalencia de personas con DM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -665,20 +665,86 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>dm_prev_cv</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Coeficiente de variación de la prevalencia de personas con DM</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>dm2_prev</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Prevalencia de DM2 por provincia, grupo etario y sexo</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>dm2_prev_se</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Error estándar del total de la prevalencia de personas con DM2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0-Inf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>dm2_prev_cv</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Coeficiente de variación de la prevalencia de personas con DM2</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>numeric</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>0-Inf</t>
         </is>

</xml_diff>